<commit_message>
feat: add Priority, External ID, Owner, Module passthrough columns
- Add 4 optional passthrough columns to _CANONICAL_MAP and _ALIASES
- _parse_row extracts all 4 as strings (None if absent/empty)
- Fuzzy aliases: component/suite/section -> module; jira/testrailid -> external_id
- Template rebuilt with 13 columns and updated Instructions sheet
- 7 new tests in TestPassthroughColumns (224 total, all green)
</commit_message>
<xml_diff>
--- a/templates/test_suite_template.xlsx
+++ b/templates/test_suite_template.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,26 +26,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="14"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="003B5998"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -60,12 +47,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,64 +414,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Layer</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Coverage Areas</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Execution Time (secs)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Flakiness Rate</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Failure Count (30d)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Tags</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>External ID</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Module</t>
         </is>
       </c>
     </row>
@@ -532,6 +524,26 @@
           <t>critical-flow</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>JIRA-101</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>alice</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -569,6 +581,26 @@
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>JIRA-102</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>bob</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -610,6 +642,26 @@
           <t>security</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>JIRA-103</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>carol</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -647,6 +699,26 @@
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>JIRA-104</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>david</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Checkout</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -684,6 +756,18 @@
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -696,19 +780,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>SuiteCompass — Test Suite Import Template</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -779,8 +861,37 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Priority: P0/P1/P2/P3 — passthrough metadata, not used in scoring (optional)</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>External ID: Jira/TestRail/issue tracker reference e.g. JIRA-101 (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Owner: Person or team responsible for this test (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Module: Application module or component owning the test e.g. Payment, Checkout (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>After filling: run: iro import-tests tests.xlsx --output test_suite.yaml</t>
         </is>

</xml_diff>